<commit_message>
Build page lists from the query index instead of hand-authored cards
The home rails, magazine listing, adventures grid and article "Up Next"
were frozen copies of the source lists. They now resolve at runtime from
/query-index.json (index configured in the configuration service), so a
newly published article or adventure appears without editing any page.

- scripts/query-index.js: shared index loader and query (folder, template,
  tags, sort, limit, exclude) plus key/value settings detection
- cards, hero, tabs-minimal-dark-withimg: query mode when authored as
  settings rows; hand-authored rows keep working
- page-list: new block for the article "Up Next" sidebar
- importer: wknd-metadata adds Template/Tags/Date from the source page;
  wknd-dynamic-lists converts source list components to query blocks,
  inferring folder, sort, limit, exclusions and tag-based filters

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-adventure-detail.report.xlsx
+++ b/tools/importer/reports/import-adventure-detail.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="312">
   <si>
     <t>_reportFile</t>
   </si>
@@ -40,7 +40,7 @@
     <t>ca/en.report.json</t>
   </si>
   <si>
-    <t>["carousel","hero-featured-light","hero","cards","cards"]</t>
+    <t>["carousel","hero-featured-light"]</t>
   </si>
   <si>
     <t>ca/en</t>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-09-25T11:02:47.791Z</t>
+    <t>2026-09-28T06:47:37.699Z</t>
   </si>
   <si>
     <t>WKND Adventures and Travel</t>
@@ -70,7 +70,7 @@
     <t>ca/fr</t>
   </si>
   <si>
-    <t>2026-09-25T11:02:52.531Z</t>
+    <t>2026-09-28T06:47:42.443Z</t>
   </si>
   <si>
     <t>Français</t>
@@ -85,7 +85,7 @@
     <t>ch/de</t>
   </si>
   <si>
-    <t>2026-09-25T11:02:56.825Z</t>
+    <t>2026-09-28T06:47:47.732Z</t>
   </si>
   <si>
     <t>Deutsch</t>
@@ -100,7 +100,7 @@
     <t>ch/fr</t>
   </si>
   <si>
-    <t>2026-09-25T11:03:01.683Z</t>
+    <t>2026-09-28T06:47:52.944Z</t>
   </si>
   <si>
     <t>https://wknd.site/ch/fr.html</t>
@@ -112,7 +112,7 @@
     <t>ch/it</t>
   </si>
   <si>
-    <t>2026-09-25T11:03:06.466Z</t>
+    <t>2026-09-28T06:47:57.192Z</t>
   </si>
   <si>
     <t>Italiano</t>
@@ -127,7 +127,7 @@
     <t>de/de</t>
   </si>
   <si>
-    <t>2026-09-25T11:03:11.353Z</t>
+    <t>2026-09-28T06:48:03.627Z</t>
   </si>
   <si>
     <t>https://wknd.site/de/de.html</t>
@@ -139,7 +139,7 @@
     <t>es/es</t>
   </si>
   <si>
-    <t>2026-09-25T11:03:16.325Z</t>
+    <t>2026-09-28T06:48:09.290Z</t>
   </si>
   <si>
     <t>Español</t>
@@ -154,7 +154,7 @@
     <t>fr/fr</t>
   </si>
   <si>
-    <t>2026-09-25T11:03:21.861Z</t>
+    <t>2026-09-28T06:48:13.686Z</t>
   </si>
   <si>
     <t>https://wknd.site/fr/fr.html</t>
@@ -166,7 +166,7 @@
     <t>it/it</t>
   </si>
   <si>
-    <t>2026-09-25T11:03:26.927Z</t>
+    <t>2026-09-28T06:48:18.891Z</t>
   </si>
   <si>
     <t>https://wknd.site/it/it.html</t>
@@ -178,7 +178,7 @@
     <t>us/en</t>
   </si>
   <si>
-    <t>2026-09-25T11:03:31.243Z</t>
+    <t>2026-09-28T06:48:24.057Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en.html</t>
@@ -190,7 +190,7 @@
     <t>us/es</t>
   </si>
   <si>
-    <t>2026-09-25T11:03:35.709Z</t>
+    <t>2026-09-28T06:48:29.086Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/es.html</t>
@@ -208,7 +208,7 @@
     <t>content-landing</t>
   </si>
   <si>
-    <t>2026-09-25T11:03:40.337Z</t>
+    <t>2026-09-28T06:48:37.098Z</t>
   </si>
   <si>
     <t>About Us</t>
@@ -220,16 +220,13 @@
     <t>ca/en/adventures.report.json</t>
   </si>
   <si>
-    <t>["hero","tabs-minimal-dark-withimg"]</t>
-  </si>
-  <si>
     <t>ca/en/adventures</t>
   </si>
   <si>
     <t>category-listing</t>
   </si>
   <si>
-    <t>2026-09-25T11:04:09.164Z</t>
+    <t>2026-09-28T06:49:07.860Z</t>
   </si>
   <si>
     <t>Adventures</t>
@@ -250,7 +247,7 @@
     <t>faq-page</t>
   </si>
   <si>
-    <t>2026-09-25T11:04:19.230Z</t>
+    <t>2026-09-28T06:49:22.059Z</t>
   </si>
   <si>
     <t>FAQs</t>
@@ -268,7 +265,7 @@
     <t>ca/en/magazine</t>
   </si>
   <si>
-    <t>2026-09-25T11:03:45.964Z</t>
+    <t>2026-09-28T06:48:43.457Z</t>
   </si>
   <si>
     <t>Magazine</t>
@@ -283,7 +280,7 @@
     <t>us/en/about-us</t>
   </si>
   <si>
-    <t>2026-09-25T11:03:57.560Z</t>
+    <t>2026-09-28T06:48:54.077Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/about-us.html</t>
@@ -295,7 +292,7 @@
     <t>us/en/adventures</t>
   </si>
   <si>
-    <t>2026-09-25T11:04:13.434Z</t>
+    <t>2026-09-28T06:49:13.949Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures.html</t>
@@ -307,7 +304,7 @@
     <t>us/en/faqs</t>
   </si>
   <si>
-    <t>2026-09-25T11:04:24.945Z</t>
+    <t>2026-09-28T06:49:27.728Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/faqs.html</t>
@@ -319,7 +316,7 @@
     <t>us/en/magazine</t>
   </si>
   <si>
-    <t>2026-09-25T11:04:03.171Z</t>
+    <t>2026-09-28T06:48:59.826Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/magazine.html</t>
@@ -337,7 +334,7 @@
     <t>adventure-detail</t>
   </si>
   <si>
-    <t>2026-09-25T11:05:35.675Z</t>
+    <t>2026-09-28T06:50:43.640Z</t>
   </si>
   <si>
     <t>Bali Surf Camp</t>
@@ -352,7 +349,7 @@
     <t>ca/en/adventures/beervana-portland</t>
   </si>
   <si>
-    <t>2026-09-25T11:05:40.051Z</t>
+    <t>2026-09-28T06:50:49.350Z</t>
   </si>
   <si>
     <t>Beervana in Portland</t>
@@ -367,7 +364,7 @@
     <t>ca/en/adventures/climbing-new-zealand</t>
   </si>
   <si>
-    <t>2026-09-25T11:05:46.255Z</t>
+    <t>2026-09-28T06:50:54.837Z</t>
   </si>
   <si>
     <t>Climbing New Zealand</t>
@@ -382,7 +379,7 @@
     <t>ca/en/adventures/colorado-rock-climbing</t>
   </si>
   <si>
-    <t>2026-09-25T11:05:50.486Z</t>
+    <t>2026-09-28T06:51:00.599Z</t>
   </si>
   <si>
     <t>Colorado Rock Climbing</t>
@@ -397,7 +394,7 @@
     <t>ca/en/adventures/cycling-southern-utah</t>
   </si>
   <si>
-    <t>2026-09-25T11:05:55.526Z</t>
+    <t>2026-09-28T06:51:05.101Z</t>
   </si>
   <si>
     <t>Cycling Southern Utah</t>
@@ -412,7 +409,7 @@
     <t>ca/en/adventures/cycling-tuscany</t>
   </si>
   <si>
-    <t>2026-09-25T11:05:59.990Z</t>
+    <t>2026-09-28T06:51:10.772Z</t>
   </si>
   <si>
     <t>Cycling Tuscany</t>
@@ -427,7 +424,7 @@
     <t>ca/en/adventures/downhill-skiing-wyoming</t>
   </si>
   <si>
-    <t>2026-09-25T11:06:04.362Z</t>
+    <t>2026-09-28T06:51:15.715Z</t>
   </si>
   <si>
     <t>Downhill Skiing Wyoming</t>
@@ -442,7 +439,7 @@
     <t>ca/en/adventures/gastronomic-marais-tour</t>
   </si>
   <si>
-    <t>2026-09-25T11:06:09.141Z</t>
+    <t>2026-09-28T06:51:19.918Z</t>
   </si>
   <si>
     <t>Gastronomic Marais Tour</t>
@@ -457,7 +454,7 @@
     <t>ca/en/adventures/napa-wine-tasting</t>
   </si>
   <si>
-    <t>2026-09-25T11:06:13.935Z</t>
+    <t>2026-09-28T06:51:25.955Z</t>
   </si>
   <si>
     <t>Napa Wine Tasting</t>
@@ -472,7 +469,7 @@
     <t>ca/en/adventures/riverside-camping-australia</t>
   </si>
   <si>
-    <t>2026-09-25T11:06:19.300Z</t>
+    <t>2026-09-28T06:51:30.399Z</t>
   </si>
   <si>
     <t>Riverside Camping</t>
@@ -487,7 +484,7 @@
     <t>ca/en/adventures/ski-touring-mont-blanc</t>
   </si>
   <si>
-    <t>2026-09-25T11:06:26.397Z</t>
+    <t>2026-09-28T06:51:34.955Z</t>
   </si>
   <si>
     <t>Ski Touring Mont Blanc</t>
@@ -502,7 +499,7 @@
     <t>ca/en/adventures/surf-camp-costa-rica</t>
   </si>
   <si>
-    <t>2026-09-25T11:06:32.405Z</t>
+    <t>2026-09-28T06:51:40.370Z</t>
   </si>
   <si>
     <t>Surf Camp in Costa Rica</t>
@@ -517,7 +514,7 @@
     <t>ca/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-09-25T11:06:38.802Z</t>
+    <t>2026-09-28T06:51:46.152Z</t>
   </si>
   <si>
     <t>Tahoe Skiing</t>
@@ -532,7 +529,7 @@
     <t>ca/en/adventures/west-coast-cycling</t>
   </si>
   <si>
-    <t>2026-09-25T11:06:44.060Z</t>
+    <t>2026-09-28T06:51:51.448Z</t>
   </si>
   <si>
     <t>West Coast Cycling</t>
@@ -547,7 +544,7 @@
     <t>ca/en/adventures/whistler-mountain-biking</t>
   </si>
   <si>
-    <t>2026-09-25T11:06:48.827Z</t>
+    <t>2026-09-28T06:51:56.757Z</t>
   </si>
   <si>
     <t>Whistler Mountain Biking</t>
@@ -562,7 +559,7 @@
     <t>ca/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-09-25T11:06:55.079Z</t>
+    <t>2026-09-28T06:52:01.382Z</t>
   </si>
   <si>
     <t>Yosemite Backpacking</t>
@@ -583,7 +580,7 @@
     <t>magazine-article</t>
   </si>
   <si>
-    <t>2026-09-25T11:04:29.830Z</t>
+    <t>2026-09-28T06:49:35.790Z</t>
   </si>
   <si>
     <t>Arctic Surfing</t>
@@ -598,7 +595,7 @@
     <t>ca/en/magazine/guide-la-skateparks</t>
   </si>
   <si>
-    <t>2026-09-25T11:04:34.469Z</t>
+    <t>2026-09-28T06:49:40.247Z</t>
   </si>
   <si>
     <t>Ultimate Guide to LA Skateparks</t>
@@ -613,7 +610,7 @@
     <t>ca/en/magazine/members-only</t>
   </si>
   <si>
-    <t>2026-09-25T11:03:51.701Z</t>
+    <t>2026-09-28T06:48:50.102Z</t>
   </si>
   <si>
     <t>Members Only</t>
@@ -631,7 +628,7 @@
     <t>ca/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-09-25T11:04:51.479Z</t>
+    <t>2026-09-28T06:49:56.658Z</t>
   </si>
   <si>
     <t>San Diego Surf Spots</t>
@@ -646,7 +643,7 @@
     <t>ca/en/magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-09-25T11:04:57.066Z</t>
+    <t>2026-09-28T06:50:02.602Z</t>
   </si>
   <si>
     <t>Ski Touring</t>
@@ -661,7 +658,7 @@
     <t>ca/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-09-25T11:05:03.434Z</t>
+    <t>2026-09-28T06:50:08.953Z</t>
   </si>
   <si>
     <t>Western Australia</t>
@@ -676,7 +673,7 @@
     <t>us/en/adventures/bali-surf-camp</t>
   </si>
   <si>
-    <t>2026-09-25T11:06:59.980Z</t>
+    <t>2026-09-28T06:52:06.374Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/bali-surf-camp.html</t>
@@ -688,7 +685,7 @@
     <t>us/en/adventures/beervana-portland</t>
   </si>
   <si>
-    <t>2026-09-25T11:07:05.231Z</t>
+    <t>2026-09-28T06:52:10.736Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/beervana-portland.html</t>
@@ -700,7 +697,7 @@
     <t>us/en/adventures/climbing-new-zealand</t>
   </si>
   <si>
-    <t>2026-09-25T11:07:10.528Z</t>
+    <t>2026-09-28T06:52:16.027Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/climbing-new-zealand.html</t>
@@ -712,7 +709,7 @@
     <t>us/en/adventures/colorado-rock-climbing</t>
   </si>
   <si>
-    <t>2026-09-25T11:07:15.226Z</t>
+    <t>2026-09-28T06:52:21.755Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/colorado-rock-climbing.html</t>
@@ -724,7 +721,7 @@
     <t>us/en/adventures/cycling-southern-utah</t>
   </si>
   <si>
-    <t>2026-09-25T11:07:19.826Z</t>
+    <t>2026-09-28T06:52:27.095Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/cycling-southern-utah.html</t>
@@ -736,7 +733,7 @@
     <t>us/en/adventures/cycling-tuscany</t>
   </si>
   <si>
-    <t>2026-09-25T11:07:24.800Z</t>
+    <t>2026-09-28T06:52:32.934Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/cycling-tuscany.html</t>
@@ -748,7 +745,7 @@
     <t>us/en/adventures/downhill-skiing-wyoming</t>
   </si>
   <si>
-    <t>2026-09-25T11:07:30.069Z</t>
+    <t>2026-09-28T06:52:38.326Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/downhill-skiing-wyoming.html</t>
@@ -760,7 +757,7 @@
     <t>us/en/adventures/gastronomic-marais-tour</t>
   </si>
   <si>
-    <t>2026-09-25T11:07:34.932Z</t>
+    <t>2026-09-28T06:52:43.365Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/gastronomic-marais-tour.html</t>
@@ -772,7 +769,7 @@
     <t>us/en/adventures/napa-wine-tasting</t>
   </si>
   <si>
-    <t>2026-09-25T11:07:40.547Z</t>
+    <t>2026-09-28T06:52:49.503Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/napa-wine-tasting.html</t>
@@ -784,7 +781,7 @@
     <t>us/en/adventures/riverside-camping-australia</t>
   </si>
   <si>
-    <t>2026-09-25T11:07:46.293Z</t>
+    <t>2026-09-28T06:52:53.649Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/riverside-camping-australia.html</t>
@@ -796,7 +793,7 @@
     <t>us/en/adventures/ski-touring-mont-blanc</t>
   </si>
   <si>
-    <t>2026-09-25T11:07:50.532Z</t>
+    <t>2026-09-28T06:52:59.412Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/ski-touring-mont-blanc.html</t>
@@ -808,7 +805,7 @@
     <t>us/en/adventures/surf-camp-costa-rica</t>
   </si>
   <si>
-    <t>2026-09-25T11:07:55.297Z</t>
+    <t>2026-09-28T06:53:04.795Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/surf-camp-costa-rica.html</t>
@@ -820,7 +817,7 @@
     <t>us/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-09-25T11:08:00.164Z</t>
+    <t>2026-09-28T06:53:10.008Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/tahoe-skiing.html</t>
@@ -832,7 +829,7 @@
     <t>us/en/adventures/west-coast-cycling</t>
   </si>
   <si>
-    <t>2026-09-25T11:08:04.879Z</t>
+    <t>2026-09-28T06:53:15.333Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/west-coast-cycling.html</t>
@@ -844,7 +841,7 @@
     <t>us/en/adventures/whistler-mountain-biking</t>
   </si>
   <si>
-    <t>2026-09-25T11:08:10.137Z</t>
+    <t>2026-09-28T06:53:20.566Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/whistler-mountain-biking.html</t>
@@ -856,7 +853,7 @@
     <t>us/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-09-25T11:08:14.443Z</t>
+    <t>2026-09-28T06:53:26.426Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/yosemite-backpacking.html</t>
@@ -868,7 +865,7 @@
     <t>us/en/magazine/arctic-surfing</t>
   </si>
   <si>
-    <t>2026-09-25T11:05:09.651Z</t>
+    <t>2026-09-28T06:50:12.935Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/magazine/arctic-surfing.html</t>
@@ -880,7 +877,7 @@
     <t>us/en/magazine/guide-la-skateparks</t>
   </si>
   <si>
-    <t>2026-09-25T11:05:15.669Z</t>
+    <t>2026-09-28T06:50:18.371Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/magazine/guide-la-skateparks.html</t>
@@ -892,7 +889,7 @@
     <t>us/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-09-25T11:05:21.387Z</t>
+    <t>2026-09-28T06:50:24.350Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/magazine/san-diego-surf.html</t>
@@ -904,7 +901,7 @@
     <t>us/en/magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-09-25T11:05:26.066Z</t>
+    <t>2026-09-28T06:50:30.110Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/magazine/ski-touring.html</t>
@@ -916,7 +913,7 @@
     <t>us/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-09-25T11:05:30.065Z</t>
+    <t>2026-09-28T06:50:35.893Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/magazine/western-australia.html</t>
@@ -928,7 +925,7 @@
     <t>ca/en/magazine/members-only/alaskan-adventure</t>
   </si>
   <si>
-    <t>2026-09-25T11:04:39.216Z</t>
+    <t>2026-09-28T06:49:44.811Z</t>
   </si>
   <si>
     <t>Alaskan Adventure</t>
@@ -943,7 +940,7 @@
     <t>ca/en/magazine/members-only/fly-fishing-the-amazon</t>
   </si>
   <si>
-    <t>2026-09-25T11:04:45.387Z</t>
+    <t>2026-09-28T06:49:50.501Z</t>
   </si>
   <si>
     <t>Fly Fishing the Amazon</t>
@@ -1691,62 +1688,62 @@
         <v>68</v>
       </c>
       <c r="B14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" t="s">
         <v>69</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
         <v>70</v>
       </c>
-      <c r="D14" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>71</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>72</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>73</v>
-      </c>
-      <c r="H14" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>74</v>
+      </c>
+      <c r="B15" t="s">
         <v>75</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>76</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
         <v>77</v>
       </c>
-      <c r="D15" t="s">
-        <v>11</v>
-      </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>78</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>79</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>80</v>
-      </c>
-      <c r="H15" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>81</v>
+      </c>
+      <c r="B16" t="s">
         <v>82</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>83</v>
-      </c>
-      <c r="C16" t="s">
-        <v>84</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
@@ -1755,24 +1752,24 @@
         <v>64</v>
       </c>
       <c r="F16" t="s">
+        <v>84</v>
+      </c>
+      <c r="G16" t="s">
         <v>85</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>86</v>
-      </c>
-      <c r="H16" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B17" t="s">
         <v>62</v>
       </c>
       <c r="C17" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D17" t="s">
         <v>11</v>
@@ -1781,76 +1778,76 @@
         <v>64</v>
       </c>
       <c r="F17" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G17" t="s">
         <v>66</v>
       </c>
       <c r="H17" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>91</v>
+      </c>
+      <c r="B18" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" t="s">
         <v>92</v>
       </c>
-      <c r="B18" t="s">
-        <v>69</v>
-      </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
+        <v>70</v>
+      </c>
+      <c r="F18" t="s">
         <v>93</v>
       </c>
-      <c r="D18" t="s">
-        <v>11</v>
-      </c>
-      <c r="E18" t="s">
-        <v>71</v>
-      </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
+        <v>72</v>
+      </c>
+      <c r="H18" t="s">
         <v>94</v>
-      </c>
-      <c r="G18" t="s">
-        <v>73</v>
-      </c>
-      <c r="H18" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>95</v>
+      </c>
+      <c r="B19" t="s">
+        <v>75</v>
+      </c>
+      <c r="C19" t="s">
         <v>96</v>
       </c>
-      <c r="B19" t="s">
-        <v>76</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" t="s">
+        <v>77</v>
+      </c>
+      <c r="F19" t="s">
         <v>97</v>
       </c>
-      <c r="D19" t="s">
-        <v>11</v>
-      </c>
-      <c r="E19" t="s">
-        <v>78</v>
-      </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
+        <v>79</v>
+      </c>
+      <c r="H19" t="s">
         <v>98</v>
-      </c>
-      <c r="G19" t="s">
-        <v>80</v>
-      </c>
-      <c r="H19" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>99</v>
+      </c>
+      <c r="B20" t="s">
+        <v>82</v>
+      </c>
+      <c r="C20" t="s">
         <v>100</v>
-      </c>
-      <c r="B20" t="s">
-        <v>83</v>
-      </c>
-      <c r="C20" t="s">
-        <v>101</v>
       </c>
       <c r="D20" t="s">
         <v>11</v>
@@ -1859,492 +1856,492 @@
         <v>64</v>
       </c>
       <c r="F20" t="s">
+        <v>101</v>
+      </c>
+      <c r="G20" t="s">
+        <v>85</v>
+      </c>
+      <c r="H20" t="s">
         <v>102</v>
-      </c>
-      <c r="G20" t="s">
-        <v>86</v>
-      </c>
-      <c r="H20" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B21" t="s">
+        <v>104</v>
+      </c>
+      <c r="C21" t="s">
         <v>105</v>
       </c>
-      <c r="C21" t="s">
-        <v>106</v>
-      </c>
       <c r="D21" t="s">
         <v>11</v>
       </c>
       <c r="E21" t="s">
+        <v>106</v>
+      </c>
+      <c r="F21" t="s">
         <v>107</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>108</v>
       </c>
-      <c r="G21" t="s">
+      <c r="H21" t="s">
         <v>109</v>
-      </c>
-      <c r="H21" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>110</v>
+      </c>
+      <c r="B22" t="s">
+        <v>104</v>
+      </c>
+      <c r="C22" t="s">
         <v>111</v>
       </c>
-      <c r="B22" t="s">
-        <v>105</v>
-      </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" t="s">
+        <v>106</v>
+      </c>
+      <c r="F22" t="s">
         <v>112</v>
       </c>
-      <c r="D22" t="s">
-        <v>11</v>
-      </c>
-      <c r="E22" t="s">
-        <v>107</v>
-      </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>113</v>
       </c>
-      <c r="G22" t="s">
+      <c r="H22" t="s">
         <v>114</v>
-      </c>
-      <c r="H22" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>115</v>
+      </c>
+      <c r="B23" t="s">
+        <v>104</v>
+      </c>
+      <c r="C23" t="s">
         <v>116</v>
       </c>
-      <c r="B23" t="s">
-        <v>105</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" t="s">
+        <v>106</v>
+      </c>
+      <c r="F23" t="s">
         <v>117</v>
       </c>
-      <c r="D23" t="s">
-        <v>11</v>
-      </c>
-      <c r="E23" t="s">
-        <v>107</v>
-      </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>118</v>
       </c>
-      <c r="G23" t="s">
+      <c r="H23" t="s">
         <v>119</v>
-      </c>
-      <c r="H23" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>120</v>
+      </c>
+      <c r="B24" t="s">
+        <v>104</v>
+      </c>
+      <c r="C24" t="s">
         <v>121</v>
       </c>
-      <c r="B24" t="s">
-        <v>105</v>
-      </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" t="s">
+        <v>106</v>
+      </c>
+      <c r="F24" t="s">
         <v>122</v>
       </c>
-      <c r="D24" t="s">
-        <v>11</v>
-      </c>
-      <c r="E24" t="s">
-        <v>107</v>
-      </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
         <v>123</v>
       </c>
-      <c r="G24" t="s">
+      <c r="H24" t="s">
         <v>124</v>
-      </c>
-      <c r="H24" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>125</v>
+      </c>
+      <c r="B25" t="s">
+        <v>104</v>
+      </c>
+      <c r="C25" t="s">
         <v>126</v>
       </c>
-      <c r="B25" t="s">
-        <v>105</v>
-      </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
+        <v>11</v>
+      </c>
+      <c r="E25" t="s">
+        <v>106</v>
+      </c>
+      <c r="F25" t="s">
         <v>127</v>
       </c>
-      <c r="D25" t="s">
-        <v>11</v>
-      </c>
-      <c r="E25" t="s">
-        <v>107</v>
-      </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
         <v>128</v>
       </c>
-      <c r="G25" t="s">
+      <c r="H25" t="s">
         <v>129</v>
-      </c>
-      <c r="H25" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>130</v>
+      </c>
+      <c r="B26" t="s">
+        <v>104</v>
+      </c>
+      <c r="C26" t="s">
         <v>131</v>
       </c>
-      <c r="B26" t="s">
-        <v>105</v>
-      </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" t="s">
+        <v>106</v>
+      </c>
+      <c r="F26" t="s">
         <v>132</v>
       </c>
-      <c r="D26" t="s">
-        <v>11</v>
-      </c>
-      <c r="E26" t="s">
-        <v>107</v>
-      </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
         <v>133</v>
       </c>
-      <c r="G26" t="s">
+      <c r="H26" t="s">
         <v>134</v>
-      </c>
-      <c r="H26" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>135</v>
+      </c>
+      <c r="B27" t="s">
+        <v>104</v>
+      </c>
+      <c r="C27" t="s">
         <v>136</v>
       </c>
-      <c r="B27" t="s">
-        <v>105</v>
-      </c>
-      <c r="C27" t="s">
+      <c r="D27" t="s">
+        <v>11</v>
+      </c>
+      <c r="E27" t="s">
+        <v>106</v>
+      </c>
+      <c r="F27" t="s">
         <v>137</v>
       </c>
-      <c r="D27" t="s">
-        <v>11</v>
-      </c>
-      <c r="E27" t="s">
-        <v>107</v>
-      </c>
-      <c r="F27" t="s">
+      <c r="G27" t="s">
         <v>138</v>
       </c>
-      <c r="G27" t="s">
+      <c r="H27" t="s">
         <v>139</v>
-      </c>
-      <c r="H27" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>140</v>
+      </c>
+      <c r="B28" t="s">
+        <v>104</v>
+      </c>
+      <c r="C28" t="s">
         <v>141</v>
       </c>
-      <c r="B28" t="s">
-        <v>105</v>
-      </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
+        <v>11</v>
+      </c>
+      <c r="E28" t="s">
+        <v>106</v>
+      </c>
+      <c r="F28" t="s">
         <v>142</v>
       </c>
-      <c r="D28" t="s">
-        <v>11</v>
-      </c>
-      <c r="E28" t="s">
-        <v>107</v>
-      </c>
-      <c r="F28" t="s">
+      <c r="G28" t="s">
         <v>143</v>
       </c>
-      <c r="G28" t="s">
+      <c r="H28" t="s">
         <v>144</v>
-      </c>
-      <c r="H28" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>145</v>
+      </c>
+      <c r="B29" t="s">
+        <v>104</v>
+      </c>
+      <c r="C29" t="s">
         <v>146</v>
       </c>
-      <c r="B29" t="s">
-        <v>105</v>
-      </c>
-      <c r="C29" t="s">
+      <c r="D29" t="s">
+        <v>11</v>
+      </c>
+      <c r="E29" t="s">
+        <v>106</v>
+      </c>
+      <c r="F29" t="s">
         <v>147</v>
       </c>
-      <c r="D29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E29" t="s">
-        <v>107</v>
-      </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
         <v>148</v>
       </c>
-      <c r="G29" t="s">
+      <c r="H29" t="s">
         <v>149</v>
-      </c>
-      <c r="H29" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>150</v>
+      </c>
+      <c r="B30" t="s">
+        <v>104</v>
+      </c>
+      <c r="C30" t="s">
         <v>151</v>
       </c>
-      <c r="B30" t="s">
-        <v>105</v>
-      </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
+        <v>11</v>
+      </c>
+      <c r="E30" t="s">
+        <v>106</v>
+      </c>
+      <c r="F30" t="s">
         <v>152</v>
       </c>
-      <c r="D30" t="s">
-        <v>11</v>
-      </c>
-      <c r="E30" t="s">
-        <v>107</v>
-      </c>
-      <c r="F30" t="s">
+      <c r="G30" t="s">
         <v>153</v>
       </c>
-      <c r="G30" t="s">
+      <c r="H30" t="s">
         <v>154</v>
-      </c>
-      <c r="H30" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>155</v>
+      </c>
+      <c r="B31" t="s">
+        <v>104</v>
+      </c>
+      <c r="C31" t="s">
         <v>156</v>
       </c>
-      <c r="B31" t="s">
-        <v>105</v>
-      </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
+        <v>11</v>
+      </c>
+      <c r="E31" t="s">
+        <v>106</v>
+      </c>
+      <c r="F31" t="s">
         <v>157</v>
       </c>
-      <c r="D31" t="s">
-        <v>11</v>
-      </c>
-      <c r="E31" t="s">
-        <v>107</v>
-      </c>
-      <c r="F31" t="s">
+      <c r="G31" t="s">
         <v>158</v>
       </c>
-      <c r="G31" t="s">
+      <c r="H31" t="s">
         <v>159</v>
-      </c>
-      <c r="H31" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>160</v>
+      </c>
+      <c r="B32" t="s">
+        <v>104</v>
+      </c>
+      <c r="C32" t="s">
         <v>161</v>
       </c>
-      <c r="B32" t="s">
-        <v>105</v>
-      </c>
-      <c r="C32" t="s">
+      <c r="D32" t="s">
+        <v>11</v>
+      </c>
+      <c r="E32" t="s">
+        <v>106</v>
+      </c>
+      <c r="F32" t="s">
         <v>162</v>
       </c>
-      <c r="D32" t="s">
-        <v>11</v>
-      </c>
-      <c r="E32" t="s">
-        <v>107</v>
-      </c>
-      <c r="F32" t="s">
+      <c r="G32" t="s">
         <v>163</v>
       </c>
-      <c r="G32" t="s">
+      <c r="H32" t="s">
         <v>164</v>
-      </c>
-      <c r="H32" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>165</v>
+      </c>
+      <c r="B33" t="s">
+        <v>104</v>
+      </c>
+      <c r="C33" t="s">
         <v>166</v>
       </c>
-      <c r="B33" t="s">
-        <v>105</v>
-      </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
+        <v>11</v>
+      </c>
+      <c r="E33" t="s">
+        <v>106</v>
+      </c>
+      <c r="F33" t="s">
         <v>167</v>
       </c>
-      <c r="D33" t="s">
-        <v>11</v>
-      </c>
-      <c r="E33" t="s">
-        <v>107</v>
-      </c>
-      <c r="F33" t="s">
+      <c r="G33" t="s">
         <v>168</v>
       </c>
-      <c r="G33" t="s">
+      <c r="H33" t="s">
         <v>169</v>
-      </c>
-      <c r="H33" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>170</v>
+      </c>
+      <c r="B34" t="s">
+        <v>104</v>
+      </c>
+      <c r="C34" t="s">
         <v>171</v>
       </c>
-      <c r="B34" t="s">
-        <v>105</v>
-      </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
+        <v>11</v>
+      </c>
+      <c r="E34" t="s">
+        <v>106</v>
+      </c>
+      <c r="F34" t="s">
         <v>172</v>
       </c>
-      <c r="D34" t="s">
-        <v>11</v>
-      </c>
-      <c r="E34" t="s">
-        <v>107</v>
-      </c>
-      <c r="F34" t="s">
+      <c r="G34" t="s">
         <v>173</v>
       </c>
-      <c r="G34" t="s">
+      <c r="H34" t="s">
         <v>174</v>
-      </c>
-      <c r="H34" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>175</v>
+      </c>
+      <c r="B35" t="s">
+        <v>104</v>
+      </c>
+      <c r="C35" t="s">
         <v>176</v>
       </c>
-      <c r="B35" t="s">
-        <v>105</v>
-      </c>
-      <c r="C35" t="s">
+      <c r="D35" t="s">
+        <v>11</v>
+      </c>
+      <c r="E35" t="s">
+        <v>106</v>
+      </c>
+      <c r="F35" t="s">
         <v>177</v>
       </c>
-      <c r="D35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E35" t="s">
-        <v>107</v>
-      </c>
-      <c r="F35" t="s">
+      <c r="G35" t="s">
         <v>178</v>
       </c>
-      <c r="G35" t="s">
+      <c r="H35" t="s">
         <v>179</v>
-      </c>
-      <c r="H35" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>180</v>
+      </c>
+      <c r="B36" t="s">
+        <v>104</v>
+      </c>
+      <c r="C36" t="s">
         <v>181</v>
       </c>
-      <c r="B36" t="s">
-        <v>105</v>
-      </c>
-      <c r="C36" t="s">
+      <c r="D36" t="s">
+        <v>11</v>
+      </c>
+      <c r="E36" t="s">
+        <v>106</v>
+      </c>
+      <c r="F36" t="s">
         <v>182</v>
       </c>
-      <c r="D36" t="s">
-        <v>11</v>
-      </c>
-      <c r="E36" t="s">
-        <v>107</v>
-      </c>
-      <c r="F36" t="s">
+      <c r="G36" t="s">
         <v>183</v>
       </c>
-      <c r="G36" t="s">
+      <c r="H36" t="s">
         <v>184</v>
-      </c>
-      <c r="H36" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>185</v>
+      </c>
+      <c r="B37" t="s">
         <v>186</v>
       </c>
-      <c r="B37" t="s">
+      <c r="C37" t="s">
         <v>187</v>
       </c>
-      <c r="C37" t="s">
+      <c r="D37" t="s">
+        <v>11</v>
+      </c>
+      <c r="E37" t="s">
         <v>188</v>
       </c>
-      <c r="D37" t="s">
-        <v>11</v>
-      </c>
-      <c r="E37" t="s">
+      <c r="F37" t="s">
         <v>189</v>
       </c>
-      <c r="F37" t="s">
+      <c r="G37" t="s">
         <v>190</v>
       </c>
-      <c r="G37" t="s">
+      <c r="H37" t="s">
         <v>191</v>
-      </c>
-      <c r="H37" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>192</v>
+      </c>
+      <c r="B38" t="s">
+        <v>186</v>
+      </c>
+      <c r="C38" t="s">
         <v>193</v>
       </c>
-      <c r="B38" t="s">
-        <v>187</v>
-      </c>
-      <c r="C38" t="s">
+      <c r="D38" t="s">
+        <v>11</v>
+      </c>
+      <c r="E38" t="s">
+        <v>188</v>
+      </c>
+      <c r="F38" t="s">
         <v>194</v>
       </c>
-      <c r="D38" t="s">
-        <v>11</v>
-      </c>
-      <c r="E38" t="s">
-        <v>189</v>
-      </c>
-      <c r="F38" t="s">
+      <c r="G38" t="s">
         <v>195</v>
       </c>
-      <c r="G38" t="s">
+      <c r="H38" t="s">
         <v>196</v>
-      </c>
-      <c r="H38" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>197</v>
+      </c>
+      <c r="B39" t="s">
+        <v>82</v>
+      </c>
+      <c r="C39" t="s">
         <v>198</v>
-      </c>
-      <c r="B39" t="s">
-        <v>83</v>
-      </c>
-      <c r="C39" t="s">
-        <v>199</v>
       </c>
       <c r="D39" t="s">
         <v>11</v>
@@ -2353,689 +2350,689 @@
         <v>64</v>
       </c>
       <c r="F39" t="s">
+        <v>199</v>
+      </c>
+      <c r="G39" t="s">
         <v>200</v>
       </c>
-      <c r="G39" t="s">
+      <c r="H39" t="s">
         <v>201</v>
-      </c>
-      <c r="H39" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>202</v>
+      </c>
+      <c r="B40" t="s">
         <v>203</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C40" t="s">
         <v>204</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D40" t="s">
+        <v>11</v>
+      </c>
+      <c r="E40" t="s">
+        <v>188</v>
+      </c>
+      <c r="F40" t="s">
         <v>205</v>
       </c>
-      <c r="D40" t="s">
-        <v>11</v>
-      </c>
-      <c r="E40" t="s">
-        <v>189</v>
-      </c>
-      <c r="F40" t="s">
+      <c r="G40" t="s">
         <v>206</v>
       </c>
-      <c r="G40" t="s">
+      <c r="H40" t="s">
         <v>207</v>
-      </c>
-      <c r="H40" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>208</v>
+      </c>
+      <c r="B41" t="s">
+        <v>186</v>
+      </c>
+      <c r="C41" t="s">
         <v>209</v>
       </c>
-      <c r="B41" t="s">
-        <v>187</v>
-      </c>
-      <c r="C41" t="s">
+      <c r="D41" t="s">
+        <v>11</v>
+      </c>
+      <c r="E41" t="s">
+        <v>188</v>
+      </c>
+      <c r="F41" t="s">
         <v>210</v>
       </c>
-      <c r="D41" t="s">
-        <v>11</v>
-      </c>
-      <c r="E41" t="s">
-        <v>189</v>
-      </c>
-      <c r="F41" t="s">
+      <c r="G41" t="s">
         <v>211</v>
       </c>
-      <c r="G41" t="s">
+      <c r="H41" t="s">
         <v>212</v>
-      </c>
-      <c r="H41" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>213</v>
+      </c>
+      <c r="B42" t="s">
+        <v>186</v>
+      </c>
+      <c r="C42" t="s">
         <v>214</v>
       </c>
-      <c r="B42" t="s">
-        <v>187</v>
-      </c>
-      <c r="C42" t="s">
+      <c r="D42" t="s">
+        <v>11</v>
+      </c>
+      <c r="E42" t="s">
+        <v>188</v>
+      </c>
+      <c r="F42" t="s">
         <v>215</v>
       </c>
-      <c r="D42" t="s">
-        <v>11</v>
-      </c>
-      <c r="E42" t="s">
-        <v>189</v>
-      </c>
-      <c r="F42" t="s">
+      <c r="G42" t="s">
         <v>216</v>
       </c>
-      <c r="G42" t="s">
+      <c r="H42" t="s">
         <v>217</v>
-      </c>
-      <c r="H42" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>218</v>
+      </c>
+      <c r="B43" t="s">
+        <v>104</v>
+      </c>
+      <c r="C43" t="s">
         <v>219</v>
       </c>
-      <c r="B43" t="s">
-        <v>105</v>
-      </c>
-      <c r="C43" t="s">
+      <c r="D43" t="s">
+        <v>11</v>
+      </c>
+      <c r="E43" t="s">
+        <v>106</v>
+      </c>
+      <c r="F43" t="s">
         <v>220</v>
       </c>
-      <c r="D43" t="s">
-        <v>11</v>
-      </c>
-      <c r="E43" t="s">
-        <v>107</v>
-      </c>
-      <c r="F43" t="s">
+      <c r="G43" t="s">
+        <v>108</v>
+      </c>
+      <c r="H43" t="s">
         <v>221</v>
-      </c>
-      <c r="G43" t="s">
-        <v>109</v>
-      </c>
-      <c r="H43" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>222</v>
+      </c>
+      <c r="B44" t="s">
+        <v>104</v>
+      </c>
+      <c r="C44" t="s">
         <v>223</v>
       </c>
-      <c r="B44" t="s">
-        <v>105</v>
-      </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
+        <v>11</v>
+      </c>
+      <c r="E44" t="s">
+        <v>106</v>
+      </c>
+      <c r="F44" t="s">
         <v>224</v>
       </c>
-      <c r="D44" t="s">
-        <v>11</v>
-      </c>
-      <c r="E44" t="s">
-        <v>107</v>
-      </c>
-      <c r="F44" t="s">
+      <c r="G44" t="s">
+        <v>113</v>
+      </c>
+      <c r="H44" t="s">
         <v>225</v>
-      </c>
-      <c r="G44" t="s">
-        <v>114</v>
-      </c>
-      <c r="H44" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>226</v>
+      </c>
+      <c r="B45" t="s">
+        <v>104</v>
+      </c>
+      <c r="C45" t="s">
         <v>227</v>
       </c>
-      <c r="B45" t="s">
-        <v>105</v>
-      </c>
-      <c r="C45" t="s">
+      <c r="D45" t="s">
+        <v>11</v>
+      </c>
+      <c r="E45" t="s">
+        <v>106</v>
+      </c>
+      <c r="F45" t="s">
         <v>228</v>
       </c>
-      <c r="D45" t="s">
-        <v>11</v>
-      </c>
-      <c r="E45" t="s">
-        <v>107</v>
-      </c>
-      <c r="F45" t="s">
+      <c r="G45" t="s">
+        <v>118</v>
+      </c>
+      <c r="H45" t="s">
         <v>229</v>
-      </c>
-      <c r="G45" t="s">
-        <v>119</v>
-      </c>
-      <c r="H45" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>230</v>
+      </c>
+      <c r="B46" t="s">
+        <v>104</v>
+      </c>
+      <c r="C46" t="s">
         <v>231</v>
       </c>
-      <c r="B46" t="s">
-        <v>105</v>
-      </c>
-      <c r="C46" t="s">
+      <c r="D46" t="s">
+        <v>11</v>
+      </c>
+      <c r="E46" t="s">
+        <v>106</v>
+      </c>
+      <c r="F46" t="s">
         <v>232</v>
       </c>
-      <c r="D46" t="s">
-        <v>11</v>
-      </c>
-      <c r="E46" t="s">
-        <v>107</v>
-      </c>
-      <c r="F46" t="s">
+      <c r="G46" t="s">
+        <v>123</v>
+      </c>
+      <c r="H46" t="s">
         <v>233</v>
-      </c>
-      <c r="G46" t="s">
-        <v>124</v>
-      </c>
-      <c r="H46" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
+        <v>234</v>
+      </c>
+      <c r="B47" t="s">
+        <v>104</v>
+      </c>
+      <c r="C47" t="s">
         <v>235</v>
       </c>
-      <c r="B47" t="s">
-        <v>105</v>
-      </c>
-      <c r="C47" t="s">
+      <c r="D47" t="s">
+        <v>11</v>
+      </c>
+      <c r="E47" t="s">
+        <v>106</v>
+      </c>
+      <c r="F47" t="s">
         <v>236</v>
       </c>
-      <c r="D47" t="s">
-        <v>11</v>
-      </c>
-      <c r="E47" t="s">
-        <v>107</v>
-      </c>
-      <c r="F47" t="s">
+      <c r="G47" t="s">
+        <v>128</v>
+      </c>
+      <c r="H47" t="s">
         <v>237</v>
-      </c>
-      <c r="G47" t="s">
-        <v>129</v>
-      </c>
-      <c r="H47" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>238</v>
+      </c>
+      <c r="B48" t="s">
+        <v>104</v>
+      </c>
+      <c r="C48" t="s">
         <v>239</v>
       </c>
-      <c r="B48" t="s">
-        <v>105</v>
-      </c>
-      <c r="C48" t="s">
+      <c r="D48" t="s">
+        <v>11</v>
+      </c>
+      <c r="E48" t="s">
+        <v>106</v>
+      </c>
+      <c r="F48" t="s">
         <v>240</v>
       </c>
-      <c r="D48" t="s">
-        <v>11</v>
-      </c>
-      <c r="E48" t="s">
-        <v>107</v>
-      </c>
-      <c r="F48" t="s">
+      <c r="G48" t="s">
+        <v>133</v>
+      </c>
+      <c r="H48" t="s">
         <v>241</v>
-      </c>
-      <c r="G48" t="s">
-        <v>134</v>
-      </c>
-      <c r="H48" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>242</v>
+      </c>
+      <c r="B49" t="s">
+        <v>104</v>
+      </c>
+      <c r="C49" t="s">
         <v>243</v>
       </c>
-      <c r="B49" t="s">
-        <v>105</v>
-      </c>
-      <c r="C49" t="s">
+      <c r="D49" t="s">
+        <v>11</v>
+      </c>
+      <c r="E49" t="s">
+        <v>106</v>
+      </c>
+      <c r="F49" t="s">
         <v>244</v>
       </c>
-      <c r="D49" t="s">
-        <v>11</v>
-      </c>
-      <c r="E49" t="s">
-        <v>107</v>
-      </c>
-      <c r="F49" t="s">
+      <c r="G49" t="s">
+        <v>138</v>
+      </c>
+      <c r="H49" t="s">
         <v>245</v>
-      </c>
-      <c r="G49" t="s">
-        <v>139</v>
-      </c>
-      <c r="H49" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>246</v>
+      </c>
+      <c r="B50" t="s">
+        <v>104</v>
+      </c>
+      <c r="C50" t="s">
         <v>247</v>
       </c>
-      <c r="B50" t="s">
-        <v>105</v>
-      </c>
-      <c r="C50" t="s">
+      <c r="D50" t="s">
+        <v>11</v>
+      </c>
+      <c r="E50" t="s">
+        <v>106</v>
+      </c>
+      <c r="F50" t="s">
         <v>248</v>
       </c>
-      <c r="D50" t="s">
-        <v>11</v>
-      </c>
-      <c r="E50" t="s">
-        <v>107</v>
-      </c>
-      <c r="F50" t="s">
+      <c r="G50" t="s">
+        <v>143</v>
+      </c>
+      <c r="H50" t="s">
         <v>249</v>
-      </c>
-      <c r="G50" t="s">
-        <v>144</v>
-      </c>
-      <c r="H50" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>250</v>
+      </c>
+      <c r="B51" t="s">
+        <v>104</v>
+      </c>
+      <c r="C51" t="s">
         <v>251</v>
       </c>
-      <c r="B51" t="s">
-        <v>105</v>
-      </c>
-      <c r="C51" t="s">
+      <c r="D51" t="s">
+        <v>11</v>
+      </c>
+      <c r="E51" t="s">
+        <v>106</v>
+      </c>
+      <c r="F51" t="s">
         <v>252</v>
       </c>
-      <c r="D51" t="s">
-        <v>11</v>
-      </c>
-      <c r="E51" t="s">
-        <v>107</v>
-      </c>
-      <c r="F51" t="s">
+      <c r="G51" t="s">
+        <v>148</v>
+      </c>
+      <c r="H51" t="s">
         <v>253</v>
-      </c>
-      <c r="G51" t="s">
-        <v>149</v>
-      </c>
-      <c r="H51" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>254</v>
+      </c>
+      <c r="B52" t="s">
+        <v>104</v>
+      </c>
+      <c r="C52" t="s">
         <v>255</v>
       </c>
-      <c r="B52" t="s">
-        <v>105</v>
-      </c>
-      <c r="C52" t="s">
+      <c r="D52" t="s">
+        <v>11</v>
+      </c>
+      <c r="E52" t="s">
+        <v>106</v>
+      </c>
+      <c r="F52" t="s">
         <v>256</v>
       </c>
-      <c r="D52" t="s">
-        <v>11</v>
-      </c>
-      <c r="E52" t="s">
-        <v>107</v>
-      </c>
-      <c r="F52" t="s">
+      <c r="G52" t="s">
+        <v>153</v>
+      </c>
+      <c r="H52" t="s">
         <v>257</v>
-      </c>
-      <c r="G52" t="s">
-        <v>154</v>
-      </c>
-      <c r="H52" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>258</v>
+      </c>
+      <c r="B53" t="s">
+        <v>104</v>
+      </c>
+      <c r="C53" t="s">
         <v>259</v>
       </c>
-      <c r="B53" t="s">
-        <v>105</v>
-      </c>
-      <c r="C53" t="s">
+      <c r="D53" t="s">
+        <v>11</v>
+      </c>
+      <c r="E53" t="s">
+        <v>106</v>
+      </c>
+      <c r="F53" t="s">
         <v>260</v>
       </c>
-      <c r="D53" t="s">
-        <v>11</v>
-      </c>
-      <c r="E53" t="s">
-        <v>107</v>
-      </c>
-      <c r="F53" t="s">
+      <c r="G53" t="s">
+        <v>158</v>
+      </c>
+      <c r="H53" t="s">
         <v>261</v>
-      </c>
-      <c r="G53" t="s">
-        <v>159</v>
-      </c>
-      <c r="H53" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>262</v>
+      </c>
+      <c r="B54" t="s">
+        <v>104</v>
+      </c>
+      <c r="C54" t="s">
         <v>263</v>
       </c>
-      <c r="B54" t="s">
-        <v>105</v>
-      </c>
-      <c r="C54" t="s">
+      <c r="D54" t="s">
+        <v>11</v>
+      </c>
+      <c r="E54" t="s">
+        <v>106</v>
+      </c>
+      <c r="F54" t="s">
         <v>264</v>
       </c>
-      <c r="D54" t="s">
-        <v>11</v>
-      </c>
-      <c r="E54" t="s">
-        <v>107</v>
-      </c>
-      <c r="F54" t="s">
+      <c r="G54" t="s">
+        <v>163</v>
+      </c>
+      <c r="H54" t="s">
         <v>265</v>
-      </c>
-      <c r="G54" t="s">
-        <v>164</v>
-      </c>
-      <c r="H54" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>266</v>
+      </c>
+      <c r="B55" t="s">
+        <v>104</v>
+      </c>
+      <c r="C55" t="s">
         <v>267</v>
       </c>
-      <c r="B55" t="s">
-        <v>105</v>
-      </c>
-      <c r="C55" t="s">
+      <c r="D55" t="s">
+        <v>11</v>
+      </c>
+      <c r="E55" t="s">
+        <v>106</v>
+      </c>
+      <c r="F55" t="s">
         <v>268</v>
       </c>
-      <c r="D55" t="s">
-        <v>11</v>
-      </c>
-      <c r="E55" t="s">
-        <v>107</v>
-      </c>
-      <c r="F55" t="s">
+      <c r="G55" t="s">
+        <v>168</v>
+      </c>
+      <c r="H55" t="s">
         <v>269</v>
-      </c>
-      <c r="G55" t="s">
-        <v>169</v>
-      </c>
-      <c r="H55" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>270</v>
+      </c>
+      <c r="B56" t="s">
+        <v>104</v>
+      </c>
+      <c r="C56" t="s">
         <v>271</v>
       </c>
-      <c r="B56" t="s">
-        <v>105</v>
-      </c>
-      <c r="C56" t="s">
+      <c r="D56" t="s">
+        <v>11</v>
+      </c>
+      <c r="E56" t="s">
+        <v>106</v>
+      </c>
+      <c r="F56" t="s">
         <v>272</v>
       </c>
-      <c r="D56" t="s">
-        <v>11</v>
-      </c>
-      <c r="E56" t="s">
-        <v>107</v>
-      </c>
-      <c r="F56" t="s">
+      <c r="G56" t="s">
+        <v>173</v>
+      </c>
+      <c r="H56" t="s">
         <v>273</v>
-      </c>
-      <c r="G56" t="s">
-        <v>174</v>
-      </c>
-      <c r="H56" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
+        <v>274</v>
+      </c>
+      <c r="B57" t="s">
+        <v>104</v>
+      </c>
+      <c r="C57" t="s">
         <v>275</v>
       </c>
-      <c r="B57" t="s">
-        <v>105</v>
-      </c>
-      <c r="C57" t="s">
+      <c r="D57" t="s">
+        <v>11</v>
+      </c>
+      <c r="E57" t="s">
+        <v>106</v>
+      </c>
+      <c r="F57" t="s">
         <v>276</v>
       </c>
-      <c r="D57" t="s">
-        <v>11</v>
-      </c>
-      <c r="E57" t="s">
-        <v>107</v>
-      </c>
-      <c r="F57" t="s">
+      <c r="G57" t="s">
+        <v>178</v>
+      </c>
+      <c r="H57" t="s">
         <v>277</v>
-      </c>
-      <c r="G57" t="s">
-        <v>179</v>
-      </c>
-      <c r="H57" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
+        <v>278</v>
+      </c>
+      <c r="B58" t="s">
+        <v>104</v>
+      </c>
+      <c r="C58" t="s">
         <v>279</v>
       </c>
-      <c r="B58" t="s">
-        <v>105</v>
-      </c>
-      <c r="C58" t="s">
+      <c r="D58" t="s">
+        <v>11</v>
+      </c>
+      <c r="E58" t="s">
+        <v>106</v>
+      </c>
+      <c r="F58" t="s">
         <v>280</v>
       </c>
-      <c r="D58" t="s">
-        <v>11</v>
-      </c>
-      <c r="E58" t="s">
-        <v>107</v>
-      </c>
-      <c r="F58" t="s">
+      <c r="G58" t="s">
+        <v>183</v>
+      </c>
+      <c r="H58" t="s">
         <v>281</v>
-      </c>
-      <c r="G58" t="s">
-        <v>184</v>
-      </c>
-      <c r="H58" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
+        <v>282</v>
+      </c>
+      <c r="B59" t="s">
+        <v>186</v>
+      </c>
+      <c r="C59" t="s">
         <v>283</v>
       </c>
-      <c r="B59" t="s">
-        <v>187</v>
-      </c>
-      <c r="C59" t="s">
+      <c r="D59" t="s">
+        <v>11</v>
+      </c>
+      <c r="E59" t="s">
+        <v>188</v>
+      </c>
+      <c r="F59" t="s">
         <v>284</v>
       </c>
-      <c r="D59" t="s">
-        <v>11</v>
-      </c>
-      <c r="E59" t="s">
-        <v>189</v>
-      </c>
-      <c r="F59" t="s">
+      <c r="G59" t="s">
+        <v>190</v>
+      </c>
+      <c r="H59" t="s">
         <v>285</v>
-      </c>
-      <c r="G59" t="s">
-        <v>191</v>
-      </c>
-      <c r="H59" t="s">
-        <v>286</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>286</v>
+      </c>
+      <c r="B60" t="s">
+        <v>186</v>
+      </c>
+      <c r="C60" t="s">
         <v>287</v>
       </c>
-      <c r="B60" t="s">
-        <v>187</v>
-      </c>
-      <c r="C60" t="s">
+      <c r="D60" t="s">
+        <v>11</v>
+      </c>
+      <c r="E60" t="s">
+        <v>188</v>
+      </c>
+      <c r="F60" t="s">
         <v>288</v>
       </c>
-      <c r="D60" t="s">
-        <v>11</v>
-      </c>
-      <c r="E60" t="s">
-        <v>189</v>
-      </c>
-      <c r="F60" t="s">
+      <c r="G60" t="s">
+        <v>195</v>
+      </c>
+      <c r="H60" t="s">
         <v>289</v>
-      </c>
-      <c r="G60" t="s">
-        <v>196</v>
-      </c>
-      <c r="H60" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
+        <v>290</v>
+      </c>
+      <c r="B61" t="s">
+        <v>203</v>
+      </c>
+      <c r="C61" t="s">
         <v>291</v>
       </c>
-      <c r="B61" t="s">
-        <v>204</v>
-      </c>
-      <c r="C61" t="s">
+      <c r="D61" t="s">
+        <v>11</v>
+      </c>
+      <c r="E61" t="s">
+        <v>188</v>
+      </c>
+      <c r="F61" t="s">
         <v>292</v>
       </c>
-      <c r="D61" t="s">
-        <v>11</v>
-      </c>
-      <c r="E61" t="s">
-        <v>189</v>
-      </c>
-      <c r="F61" t="s">
+      <c r="G61" t="s">
+        <v>206</v>
+      </c>
+      <c r="H61" t="s">
         <v>293</v>
-      </c>
-      <c r="G61" t="s">
-        <v>207</v>
-      </c>
-      <c r="H61" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>294</v>
+      </c>
+      <c r="B62" t="s">
+        <v>186</v>
+      </c>
+      <c r="C62" t="s">
         <v>295</v>
       </c>
-      <c r="B62" t="s">
-        <v>187</v>
-      </c>
-      <c r="C62" t="s">
+      <c r="D62" t="s">
+        <v>11</v>
+      </c>
+      <c r="E62" t="s">
+        <v>188</v>
+      </c>
+      <c r="F62" t="s">
         <v>296</v>
       </c>
-      <c r="D62" t="s">
-        <v>11</v>
-      </c>
-      <c r="E62" t="s">
-        <v>189</v>
-      </c>
-      <c r="F62" t="s">
+      <c r="G62" t="s">
+        <v>211</v>
+      </c>
+      <c r="H62" t="s">
         <v>297</v>
-      </c>
-      <c r="G62" t="s">
-        <v>212</v>
-      </c>
-      <c r="H62" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
+        <v>298</v>
+      </c>
+      <c r="B63" t="s">
+        <v>186</v>
+      </c>
+      <c r="C63" t="s">
         <v>299</v>
       </c>
-      <c r="B63" t="s">
-        <v>187</v>
-      </c>
-      <c r="C63" t="s">
+      <c r="D63" t="s">
+        <v>11</v>
+      </c>
+      <c r="E63" t="s">
+        <v>188</v>
+      </c>
+      <c r="F63" t="s">
         <v>300</v>
       </c>
-      <c r="D63" t="s">
-        <v>11</v>
-      </c>
-      <c r="E63" t="s">
-        <v>189</v>
-      </c>
-      <c r="F63" t="s">
+      <c r="G63" t="s">
+        <v>216</v>
+      </c>
+      <c r="H63" t="s">
         <v>301</v>
-      </c>
-      <c r="G63" t="s">
-        <v>217</v>
-      </c>
-      <c r="H63" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>302</v>
+      </c>
+      <c r="B64" t="s">
+        <v>186</v>
+      </c>
+      <c r="C64" t="s">
         <v>303</v>
       </c>
-      <c r="B64" t="s">
-        <v>187</v>
-      </c>
-      <c r="C64" t="s">
+      <c r="D64" t="s">
+        <v>11</v>
+      </c>
+      <c r="E64" t="s">
+        <v>188</v>
+      </c>
+      <c r="F64" t="s">
         <v>304</v>
       </c>
-      <c r="D64" t="s">
-        <v>11</v>
-      </c>
-      <c r="E64" t="s">
-        <v>189</v>
-      </c>
-      <c r="F64" t="s">
+      <c r="G64" t="s">
         <v>305</v>
       </c>
-      <c r="G64" t="s">
+      <c r="H64" t="s">
         <v>306</v>
-      </c>
-      <c r="H64" t="s">
-        <v>307</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>307</v>
+      </c>
+      <c r="B65" t="s">
+        <v>203</v>
+      </c>
+      <c r="C65" t="s">
         <v>308</v>
       </c>
-      <c r="B65" t="s">
-        <v>204</v>
-      </c>
-      <c r="C65" t="s">
+      <c r="D65" t="s">
+        <v>11</v>
+      </c>
+      <c r="E65" t="s">
+        <v>188</v>
+      </c>
+      <c r="F65" t="s">
         <v>309</v>
       </c>
-      <c r="D65" t="s">
-        <v>11</v>
-      </c>
-      <c r="E65" t="s">
-        <v>189</v>
-      </c>
-      <c r="F65" t="s">
+      <c r="G65" t="s">
         <v>310</v>
       </c>
-      <c r="G65" t="s">
+      <c r="H65" t="s">
         <v>311</v>
-      </c>
-      <c r="H65" t="s">
-        <v>312</v>
       </c>
     </row>
   </sheetData>

</xml_diff>